<commit_message>
add/fix atomic radius graphing
</commit_message>
<xml_diff>
--- a/src/assets/081425Data.xlsx
+++ b/src/assets/081425Data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10824"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vtn2/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/vtn2/src/orbital-energy-web/src/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{D1939776-40F4-CC43-8368-5A4715EDCFE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3949E95B-85F9-3E4A-BC11-6F939FB504A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="105080" yWindow="2060" windowWidth="32720" windowHeight="18700" xr2:uid="{6FB19B8F-77AB-427E-8C06-AA7297D95998}"/>
+    <workbookView xWindow="57500" yWindow="1180" windowWidth="32720" windowHeight="18700" xr2:uid="{6FB19B8F-77AB-427E-8C06-AA7297D95998}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -70,7 +70,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="207">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="209">
   <si>
     <t>Element</t>
   </si>
@@ -692,6 +692,12 @@
   <si>
     <t>Values Copied Directly from DVG's Inorganic Textbook (Ask DVG for the name of textbook)</t>
   </si>
+  <si>
+    <t>Atomic Radius (valence) - Guerra</t>
+  </si>
+  <si>
+    <t>Atomic Radius (valence) - RDK</t>
+  </si>
 </sst>
 </file>
 
@@ -871,7 +877,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="47">
+  <cellXfs count="48">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -961,8 +967,8 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -974,6 +980,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -1380,7 +1389,9 @@
     <col min="150" max="150" width="15.1640625" style="3" bestFit="1" customWidth="1"/>
     <col min="151" max="157" width="14.5" style="3" bestFit="1" customWidth="1"/>
     <col min="158" max="158" width="15.83203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="159" max="16384" width="9.1640625" style="3"/>
+    <col min="159" max="159" width="29" style="3" bestFit="1" customWidth="1"/>
+    <col min="160" max="160" width="28.33203125" style="3" bestFit="1" customWidth="1"/>
+    <col min="161" max="16384" width="9.1640625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:214" ht="28.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
@@ -1399,44 +1410,44 @@
       <c r="J1" s="22" t="s">
         <v>187</v>
       </c>
-      <c r="K1" s="32" t="s">
+      <c r="K1" s="37" t="s">
         <v>188</v>
       </c>
-      <c r="L1" s="32"/>
-      <c r="M1" s="32"/>
-      <c r="N1" s="32"/>
-      <c r="O1" s="32"/>
-      <c r="P1" s="32"/>
-      <c r="Q1" s="32"/>
-      <c r="R1" s="32"/>
-      <c r="S1" s="32"/>
-      <c r="T1" s="32"/>
-      <c r="U1" s="32"/>
-      <c r="V1" s="32"/>
-      <c r="W1" s="32"/>
-      <c r="X1" s="32"/>
-      <c r="Y1" s="32"/>
-      <c r="Z1" s="32"/>
-      <c r="AA1" s="32"/>
-      <c r="AB1" s="32"/>
-      <c r="AC1" s="32"/>
-      <c r="AD1" s="32" t="s">
+      <c r="L1" s="37"/>
+      <c r="M1" s="37"/>
+      <c r="N1" s="37"/>
+      <c r="O1" s="37"/>
+      <c r="P1" s="37"/>
+      <c r="Q1" s="37"/>
+      <c r="R1" s="37"/>
+      <c r="S1" s="37"/>
+      <c r="T1" s="37"/>
+      <c r="U1" s="37"/>
+      <c r="V1" s="37"/>
+      <c r="W1" s="37"/>
+      <c r="X1" s="37"/>
+      <c r="Y1" s="37"/>
+      <c r="Z1" s="37"/>
+      <c r="AA1" s="37"/>
+      <c r="AB1" s="37"/>
+      <c r="AC1" s="37"/>
+      <c r="AD1" s="37" t="s">
         <v>189</v>
       </c>
-      <c r="AE1" s="32"/>
-      <c r="AF1" s="32"/>
-      <c r="AG1" s="32"/>
-      <c r="AH1" s="32"/>
-      <c r="AI1" s="32"/>
-      <c r="AJ1" s="37" t="s">
+      <c r="AE1" s="37"/>
+      <c r="AF1" s="37"/>
+      <c r="AG1" s="37"/>
+      <c r="AH1" s="37"/>
+      <c r="AI1" s="37"/>
+      <c r="AJ1" s="38" t="s">
         <v>190</v>
       </c>
-      <c r="AK1" s="38"/>
-      <c r="AL1" s="38"/>
-      <c r="AM1" s="38"/>
-      <c r="AN1" s="38"/>
-      <c r="AO1" s="39"/>
-      <c r="AP1" s="40" t="s">
+      <c r="AK1" s="39"/>
+      <c r="AL1" s="39"/>
+      <c r="AM1" s="39"/>
+      <c r="AN1" s="39"/>
+      <c r="AO1" s="40"/>
+      <c r="AP1" s="41" t="s">
         <v>191</v>
       </c>
       <c r="AQ1" s="33"/>
@@ -1457,14 +1468,14 @@
       <c r="BF1" s="33"/>
       <c r="BG1" s="33"/>
       <c r="BH1" s="33"/>
-      <c r="BI1" s="32" t="s">
+      <c r="BI1" s="37" t="s">
         <v>192</v>
       </c>
-      <c r="BJ1" s="32"/>
-      <c r="BK1" s="32"/>
-      <c r="BL1" s="32"/>
-      <c r="BM1" s="32"/>
-      <c r="BN1" s="32"/>
+      <c r="BJ1" s="37"/>
+      <c r="BK1" s="37"/>
+      <c r="BL1" s="37"/>
+      <c r="BM1" s="37"/>
+      <c r="BN1" s="37"/>
       <c r="BO1" s="22" t="s">
         <v>193</v>
       </c>
@@ -1507,72 +1518,72 @@
       <c r="CL1" s="33"/>
       <c r="CM1" s="33"/>
       <c r="CN1" s="33"/>
-      <c r="CO1" s="32" t="s">
+      <c r="CO1" s="37" t="s">
         <v>201</v>
       </c>
-      <c r="CP1" s="32"/>
-      <c r="CQ1" s="32"/>
-      <c r="CR1" s="32"/>
-      <c r="CS1" s="32"/>
-      <c r="CT1" s="32"/>
-      <c r="CU1" s="32" t="s">
+      <c r="CP1" s="37"/>
+      <c r="CQ1" s="37"/>
+      <c r="CR1" s="37"/>
+      <c r="CS1" s="37"/>
+      <c r="CT1" s="37"/>
+      <c r="CU1" s="37" t="s">
         <v>202</v>
       </c>
-      <c r="CV1" s="32"/>
-      <c r="CW1" s="32"/>
-      <c r="CX1" s="32"/>
-      <c r="CY1" s="32"/>
-      <c r="CZ1" s="32"/>
-      <c r="DA1" s="32"/>
-      <c r="DB1" s="32"/>
-      <c r="DC1" s="32"/>
-      <c r="DD1" s="32"/>
-      <c r="DE1" s="32"/>
-      <c r="DF1" s="32"/>
-      <c r="DG1" s="32"/>
-      <c r="DH1" s="32"/>
-      <c r="DI1" s="32"/>
-      <c r="DJ1" s="32"/>
-      <c r="DK1" s="32"/>
-      <c r="DL1" s="32"/>
-      <c r="DM1" s="32"/>
-      <c r="DN1" s="32" t="s">
+      <c r="CV1" s="37"/>
+      <c r="CW1" s="37"/>
+      <c r="CX1" s="37"/>
+      <c r="CY1" s="37"/>
+      <c r="CZ1" s="37"/>
+      <c r="DA1" s="37"/>
+      <c r="DB1" s="37"/>
+      <c r="DC1" s="37"/>
+      <c r="DD1" s="37"/>
+      <c r="DE1" s="37"/>
+      <c r="DF1" s="37"/>
+      <c r="DG1" s="37"/>
+      <c r="DH1" s="37"/>
+      <c r="DI1" s="37"/>
+      <c r="DJ1" s="37"/>
+      <c r="DK1" s="37"/>
+      <c r="DL1" s="37"/>
+      <c r="DM1" s="37"/>
+      <c r="DN1" s="37" t="s">
         <v>203</v>
       </c>
-      <c r="DO1" s="32"/>
-      <c r="DP1" s="32"/>
-      <c r="DQ1" s="32"/>
-      <c r="DR1" s="32"/>
-      <c r="DS1" s="32"/>
-      <c r="DT1" s="32" t="s">
+      <c r="DO1" s="37"/>
+      <c r="DP1" s="37"/>
+      <c r="DQ1" s="37"/>
+      <c r="DR1" s="37"/>
+      <c r="DS1" s="37"/>
+      <c r="DT1" s="37" t="s">
         <v>204</v>
       </c>
-      <c r="DU1" s="32"/>
-      <c r="DV1" s="32"/>
-      <c r="DW1" s="32"/>
-      <c r="DX1" s="32"/>
-      <c r="DY1" s="32"/>
-      <c r="DZ1" s="32"/>
-      <c r="EA1" s="32"/>
-      <c r="EB1" s="32"/>
-      <c r="EC1" s="32"/>
-      <c r="ED1" s="32"/>
-      <c r="EE1" s="32"/>
-      <c r="EF1" s="32"/>
-      <c r="EG1" s="32"/>
-      <c r="EH1" s="32"/>
-      <c r="EI1" s="32"/>
-      <c r="EJ1" s="32"/>
-      <c r="EK1" s="32"/>
-      <c r="EL1" s="32"/>
-      <c r="EM1" s="32" t="s">
+      <c r="DU1" s="37"/>
+      <c r="DV1" s="37"/>
+      <c r="DW1" s="37"/>
+      <c r="DX1" s="37"/>
+      <c r="DY1" s="37"/>
+      <c r="DZ1" s="37"/>
+      <c r="EA1" s="37"/>
+      <c r="EB1" s="37"/>
+      <c r="EC1" s="37"/>
+      <c r="ED1" s="37"/>
+      <c r="EE1" s="37"/>
+      <c r="EF1" s="37"/>
+      <c r="EG1" s="37"/>
+      <c r="EH1" s="37"/>
+      <c r="EI1" s="37"/>
+      <c r="EJ1" s="37"/>
+      <c r="EK1" s="37"/>
+      <c r="EL1" s="37"/>
+      <c r="EM1" s="37" t="s">
         <v>205</v>
       </c>
-      <c r="EN1" s="32"/>
-      <c r="EO1" s="32"/>
-      <c r="EP1" s="32"/>
-      <c r="EQ1" s="32"/>
-      <c r="ER1" s="32"/>
+      <c r="EN1" s="37"/>
+      <c r="EO1" s="37"/>
+      <c r="EP1" s="37"/>
+      <c r="EQ1" s="37"/>
+      <c r="ER1" s="37"/>
       <c r="ES1" s="33" t="s">
         <v>206</v>
       </c>
@@ -1759,8 +1770,12 @@
       <c r="EZ2" s="35"/>
       <c r="FA2" s="35"/>
       <c r="FB2" s="36"/>
-      <c r="FC2" s="1"/>
-      <c r="FD2" s="1"/>
+      <c r="FC2" s="1" t="s">
+        <v>207</v>
+      </c>
+      <c r="FD2" s="1" t="s">
+        <v>208</v>
+      </c>
       <c r="FE2" s="1"/>
       <c r="FF2" s="1"/>
       <c r="FG2" s="1"/>
@@ -2455,27 +2470,27 @@
       <c r="AO4" s="4" t="s">
         <v>125</v>
       </c>
-      <c r="AP4" s="41" t="s">
+      <c r="AP4" s="42" t="s">
         <v>154</v>
       </c>
-      <c r="AQ4" s="42"/>
-      <c r="AR4" s="42"/>
-      <c r="AS4" s="42"/>
-      <c r="AT4" s="42"/>
-      <c r="AU4" s="42"/>
-      <c r="AV4" s="42"/>
-      <c r="AW4" s="42"/>
-      <c r="AX4" s="42"/>
-      <c r="AY4" s="42"/>
-      <c r="AZ4" s="42"/>
-      <c r="BA4" s="42"/>
-      <c r="BB4" s="42"/>
-      <c r="BC4" s="42"/>
-      <c r="BD4" s="42"/>
-      <c r="BE4" s="42"/>
-      <c r="BF4" s="42"/>
-      <c r="BG4" s="42"/>
-      <c r="BH4" s="43"/>
+      <c r="AQ4" s="43"/>
+      <c r="AR4" s="43"/>
+      <c r="AS4" s="43"/>
+      <c r="AT4" s="43"/>
+      <c r="AU4" s="43"/>
+      <c r="AV4" s="43"/>
+      <c r="AW4" s="43"/>
+      <c r="AX4" s="43"/>
+      <c r="AY4" s="43"/>
+      <c r="AZ4" s="43"/>
+      <c r="BA4" s="43"/>
+      <c r="BB4" s="43"/>
+      <c r="BC4" s="43"/>
+      <c r="BD4" s="43"/>
+      <c r="BE4" s="43"/>
+      <c r="BF4" s="43"/>
+      <c r="BG4" s="43"/>
+      <c r="BH4" s="44"/>
       <c r="BI4" s="34" t="s">
         <v>154</v>
       </c>
@@ -2526,43 +2541,43 @@
       <c r="CL4" s="35"/>
       <c r="CM4" s="35"/>
       <c r="CN4" s="36"/>
-      <c r="CO4" s="44" t="s">
+      <c r="CO4" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="CP4" s="45"/>
-      <c r="CQ4" s="45"/>
-      <c r="CR4" s="45"/>
-      <c r="CS4" s="45"/>
-      <c r="CT4" s="46"/>
-      <c r="CU4" s="44" t="s">
+      <c r="CP4" s="46"/>
+      <c r="CQ4" s="46"/>
+      <c r="CR4" s="46"/>
+      <c r="CS4" s="46"/>
+      <c r="CT4" s="47"/>
+      <c r="CU4" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="CV4" s="45"/>
-      <c r="CW4" s="45"/>
-      <c r="CX4" s="45"/>
-      <c r="CY4" s="45"/>
-      <c r="CZ4" s="45"/>
-      <c r="DA4" s="45"/>
-      <c r="DB4" s="45"/>
-      <c r="DC4" s="45"/>
-      <c r="DD4" s="45"/>
-      <c r="DE4" s="45"/>
-      <c r="DF4" s="45"/>
-      <c r="DG4" s="45"/>
-      <c r="DH4" s="45"/>
-      <c r="DI4" s="45"/>
-      <c r="DJ4" s="45"/>
-      <c r="DK4" s="45"/>
-      <c r="DL4" s="45"/>
-      <c r="DM4" s="46"/>
-      <c r="DN4" s="44" t="s">
+      <c r="CV4" s="46"/>
+      <c r="CW4" s="46"/>
+      <c r="CX4" s="46"/>
+      <c r="CY4" s="46"/>
+      <c r="CZ4" s="46"/>
+      <c r="DA4" s="46"/>
+      <c r="DB4" s="46"/>
+      <c r="DC4" s="46"/>
+      <c r="DD4" s="46"/>
+      <c r="DE4" s="46"/>
+      <c r="DF4" s="46"/>
+      <c r="DG4" s="46"/>
+      <c r="DH4" s="46"/>
+      <c r="DI4" s="46"/>
+      <c r="DJ4" s="46"/>
+      <c r="DK4" s="46"/>
+      <c r="DL4" s="46"/>
+      <c r="DM4" s="47"/>
+      <c r="DN4" s="45" t="s">
         <v>157</v>
       </c>
-      <c r="DO4" s="45"/>
-      <c r="DP4" s="45"/>
-      <c r="DQ4" s="45"/>
-      <c r="DR4" s="45"/>
-      <c r="DS4" s="46"/>
+      <c r="DO4" s="46"/>
+      <c r="DP4" s="46"/>
+      <c r="DQ4" s="46"/>
+      <c r="DR4" s="46"/>
+      <c r="DS4" s="47"/>
       <c r="DT4" s="34" t="s">
         <v>157</v>
       </c>
@@ -2604,8 +2619,12 @@
       <c r="EZ4" s="35"/>
       <c r="FA4" s="35"/>
       <c r="FB4" s="36"/>
-      <c r="FC4" s="1"/>
-      <c r="FD4" s="1"/>
+      <c r="FC4" s="1" t="s">
+        <v>154</v>
+      </c>
+      <c r="FD4" s="1" t="s">
+        <v>154</v>
+      </c>
       <c r="FE4" s="1"/>
       <c r="FF4" s="1"/>
       <c r="FG4" s="1"/>
@@ -2815,6 +2834,12 @@
       <c r="ES5" s="3">
         <v>13.597568000000001</v>
       </c>
+      <c r="FC5" s="32">
+        <v>52.9</v>
+      </c>
+      <c r="FD5" s="16">
+        <v>52.9</v>
+      </c>
     </row>
     <row r="6" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C6" s="7" t="s">
@@ -2965,6 +2990,12 @@
       <c r="ET6" s="3">
         <v>54.415145600000002</v>
       </c>
+      <c r="FC6" s="32">
+        <v>30.152999999999995</v>
+      </c>
+      <c r="FD6" s="16">
+        <v>31.271287234714752</v>
+      </c>
     </row>
     <row r="7" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C7" s="7" t="s">
@@ -3141,6 +3172,12 @@
       <c r="EU7" s="3">
         <v>122.44962360000001</v>
       </c>
+      <c r="FC7" s="32">
+        <v>164.0429</v>
+      </c>
+      <c r="FD7" s="16">
+        <v>163.76277632628276</v>
+      </c>
     </row>
     <row r="8" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C8" s="7" t="s">
@@ -3320,6 +3357,12 @@
       <c r="EV8" s="3">
         <v>217.711366</v>
       </c>
+      <c r="FC8" s="32">
+        <v>108.4979</v>
+      </c>
+      <c r="FD8" s="16">
+        <v>105.69264919627048</v>
+      </c>
     </row>
     <row r="9" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C9" s="7" t="s">
@@ -3534,6 +3577,12 @@
       <c r="EW9" s="3">
         <v>340.21488240000002</v>
       </c>
+      <c r="FC9" s="32">
+        <v>83.952299999999994</v>
+      </c>
+      <c r="FD9" s="16">
+        <v>86.632748970302018</v>
+      </c>
     </row>
     <row r="10" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C10" s="7" t="s">
@@ -3751,6 +3800,12 @@
       <c r="EX10" s="3">
         <v>489.97779159999999</v>
       </c>
+      <c r="FC10" s="32">
+        <v>64.643799999999999</v>
+      </c>
+      <c r="FD10" s="16">
+        <v>66.815678605037164</v>
+      </c>
     </row>
     <row r="11" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C11" s="7" t="s">
@@ -3971,6 +4026,12 @@
       <c r="EY11" s="3">
         <v>667.02496720000011</v>
       </c>
+      <c r="FC11" s="32">
+        <v>54.063800000000001</v>
+      </c>
+      <c r="FD11" s="16">
+        <v>54.614604522570168</v>
+      </c>
     </row>
     <row r="12" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C12" s="7" t="s">
@@ -4194,6 +4255,12 @@
       <c r="EZ12" s="3">
         <v>871.38128280000001</v>
       </c>
+      <c r="FC12" s="32">
+        <v>46.287500000000001</v>
+      </c>
+      <c r="FD12" s="16">
+        <v>46.926099458084565</v>
+      </c>
     </row>
     <row r="13" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C13" s="7" t="s">
@@ -4420,6 +4487,12 @@
       <c r="FA13" s="3">
         <v>1103.0819760000002</v>
       </c>
+      <c r="FC13" s="32">
+        <v>40.5214</v>
+      </c>
+      <c r="FD13" s="16">
+        <v>40.932375073407002</v>
+      </c>
     </row>
     <row r="14" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C14" s="7" t="s">
@@ -4643,6 +4716,12 @@
       <c r="FB14" s="3">
         <v>1362.1550296</v>
       </c>
+      <c r="FC14" s="32">
+        <v>36.130700000000004</v>
+      </c>
+      <c r="FD14" s="16">
+        <v>36.230932694486114</v>
+      </c>
     </row>
     <row r="15" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C15" s="7" t="s">
@@ -4904,6 +4983,12 @@
       <c r="FB15" s="3">
         <v>1465.0819864</v>
       </c>
+      <c r="FC15" s="32">
+        <v>179.17230000000001</v>
+      </c>
+      <c r="FD15" s="16">
+        <v>216.94705085840147</v>
+      </c>
     </row>
     <row r="16" spans="1:214" ht="16" x14ac:dyDescent="0.2">
       <c r="C16" s="7" t="s">
@@ -5165,8 +5250,14 @@
       <c r="FB16" s="3">
         <v>367.52816800000005</v>
       </c>
+      <c r="FC16" s="32">
+        <v>136.64070000000001</v>
+      </c>
+      <c r="FD16" s="16">
+        <v>153.32226279898705</v>
+      </c>
     </row>
-    <row r="17" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="17" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C17" s="7" t="s">
         <v>13</v>
       </c>
@@ -5458,8 +5549,14 @@
       <c r="FB17" s="3">
         <v>398.56834800000001</v>
       </c>
+      <c r="FC17" s="32">
+        <v>142.03649999999999</v>
+      </c>
+      <c r="FD17" s="16">
+        <v>148.372066468935</v>
+      </c>
     </row>
-    <row r="18" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="18" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C18" s="7" t="s">
         <v>14</v>
       </c>
@@ -5751,8 +5848,14 @@
       <c r="FB18" s="3">
         <v>401.42881199999999</v>
       </c>
+      <c r="FC18" s="32">
+        <v>114.82826666666666</v>
+      </c>
+      <c r="FD18" s="16">
+        <v>115.67638265074069</v>
+      </c>
     </row>
-    <row r="19" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="19" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C19" s="7" t="s">
         <v>15</v>
       </c>
@@ -6044,8 +6147,14 @@
       <c r="FB19" s="3">
         <v>424.49907600000006</v>
       </c>
+      <c r="FC19" s="32">
+        <v>97.565233333333325</v>
+      </c>
+      <c r="FD19" s="16">
+        <v>96.080859122394756</v>
+      </c>
     </row>
-    <row r="20" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="20" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C20" s="7" t="s">
         <v>16</v>
       </c>
@@ -6337,8 +6446,14 @@
       <c r="FB20" s="3">
         <v>447.08223200000003</v>
       </c>
+      <c r="FC20" s="32">
+        <v>85.433499999999995</v>
+      </c>
+      <c r="FD20" s="16">
+        <v>83.476778810484248</v>
+      </c>
     </row>
-    <row r="21" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="21" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C21" s="7" t="s">
         <v>17</v>
       </c>
@@ -6630,8 +6745,14 @@
       <c r="FB21" s="3">
         <v>455.62216800000004</v>
       </c>
+      <c r="FC21" s="32">
+        <v>76.14073333333333</v>
+      </c>
+      <c r="FD21" s="16">
+        <v>73.664260021999198</v>
+      </c>
     </row>
-    <row r="22" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="22" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C22" s="7" t="s">
         <v>18</v>
       </c>
@@ -6917,8 +7038,14 @@
       <c r="FB22" s="3">
         <v>478.68206800000002</v>
       </c>
+      <c r="FC22" s="32">
+        <v>68.752366666666674</v>
+      </c>
+      <c r="FD22" s="16">
+        <v>66.252292761760117</v>
+      </c>
     </row>
-    <row r="23" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="23" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C23" s="7" t="s">
         <v>19</v>
       </c>
@@ -7230,8 +7357,14 @@
       <c r="FB23" s="3">
         <v>503.44166400000006</v>
       </c>
+      <c r="FC23" s="32">
+        <v>228.9512</v>
+      </c>
+      <c r="FD23" s="16">
+        <v>289.07798432468792</v>
+      </c>
     </row>
-    <row r="24" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="24" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C24" s="7" t="s">
         <v>20</v>
       </c>
@@ -7543,8 +7676,14 @@
       <c r="FB24" s="3">
         <v>211.26910359999999</v>
       </c>
+      <c r="FC24" s="32">
+        <v>183.1927</v>
+      </c>
+      <c r="FD24" s="16">
+        <v>213.50887690078227</v>
+      </c>
     </row>
-    <row r="25" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="25" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C25" s="7" t="s">
         <v>21</v>
       </c>
@@ -7763,8 +7902,12 @@
       <c r="FB25" s="3">
         <v>225.32372400000003</v>
       </c>
+      <c r="FC25" s="32">
+        <v>170.65539999999999</v>
+      </c>
+      <c r="FD25" s="16"/>
     </row>
-    <row r="26" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="26" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C26" s="7" t="s">
         <v>22</v>
       </c>
@@ -7983,8 +8126,12 @@
       <c r="FB26" s="3">
         <v>215.91321199999999</v>
       </c>
+      <c r="FC26" s="32">
+        <v>161.6095</v>
+      </c>
+      <c r="FD26" s="16"/>
     </row>
-    <row r="27" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="27" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C27" s="7" t="s">
         <v>23</v>
       </c>
@@ -8203,8 +8350,12 @@
       <c r="FB27" s="3">
         <v>230.49536000000001</v>
       </c>
+      <c r="FC27" s="32">
+        <v>154.04479999999998</v>
+      </c>
+      <c r="FD27" s="16"/>
     </row>
-    <row r="28" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="28" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C28" s="7" t="s">
         <v>24</v>
       </c>
@@ -8423,8 +8574,12 @@
       <c r="FB28" s="3">
         <v>244.38311999999999</v>
       </c>
+      <c r="FC28" s="32">
+        <v>153.83320000000001</v>
+      </c>
+      <c r="FD28" s="16"/>
     </row>
-    <row r="29" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="29" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C29" s="7" t="s">
         <v>25</v>
       </c>
@@ -8643,8 +8798,12 @@
       <c r="FB29" s="3">
         <v>248.32144000000002</v>
       </c>
+      <c r="FC29" s="32">
+        <v>141.77199999999999</v>
+      </c>
+      <c r="FD29" s="16"/>
     </row>
-    <row r="30" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="30" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C30" s="7" t="s">
         <v>26</v>
       </c>
@@ -8863,8 +9022,12 @@
       <c r="FB30" s="3">
         <v>262.10556000000003</v>
       </c>
+      <c r="FC30" s="32">
+        <v>135.79429999999999</v>
+      </c>
+      <c r="FD30" s="16"/>
     </row>
-    <row r="31" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="31" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C31" s="7" t="s">
         <v>27</v>
       </c>
@@ -9083,8 +9246,12 @@
       <c r="FB31" s="3">
         <v>275.68240000000003</v>
       </c>
+      <c r="FC31" s="32">
+        <v>130.61009999999999</v>
+      </c>
+      <c r="FD31" s="16"/>
     </row>
-    <row r="32" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="32" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C32" s="7" t="s">
         <v>28</v>
       </c>
@@ -9303,8 +9470,12 @@
       <c r="FB32" s="3">
         <v>224.48424000000003</v>
       </c>
+      <c r="FC32" s="32">
+        <v>125.95489999999998</v>
+      </c>
+      <c r="FD32" s="16"/>
     </row>
-    <row r="33" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="33" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C33" s="7" t="s">
         <v>29</v>
       </c>
@@ -9523,8 +9694,12 @@
       <c r="FB33" s="3">
         <v>232.15360000000001</v>
       </c>
+      <c r="FC33" s="32">
+        <v>134.36599999999999</v>
+      </c>
+      <c r="FD33" s="16"/>
     </row>
-    <row r="34" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="34" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C34" s="7" t="s">
         <v>30</v>
       </c>
@@ -9743,8 +9918,12 @@
       <c r="FB34" s="3">
         <v>238.37200000000001</v>
       </c>
+      <c r="FC34" s="32">
+        <v>117.80829999999999</v>
+      </c>
+      <c r="FD34" s="16"/>
     </row>
-    <row r="35" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="35" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C35" s="7" t="s">
         <v>31</v>
       </c>
@@ -9960,8 +10139,12 @@
       <c r="EV35" s="3">
         <v>64.256800000000013</v>
       </c>
+      <c r="FC35" s="32">
+        <v>138.33350000000002</v>
+      </c>
+      <c r="FD35" s="16"/>
     </row>
-    <row r="36" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="36" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C36" s="7" t="s">
         <v>32</v>
       </c>
@@ -10180,8 +10363,12 @@
       <c r="EW36" s="3">
         <v>93.483280000000008</v>
       </c>
+      <c r="FC36" s="32">
+        <v>118.98973333333333</v>
+      </c>
+      <c r="FD36" s="16"/>
     </row>
-    <row r="37" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="37" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C37" s="7" t="s">
         <v>33</v>
       </c>
@@ -10403,8 +10590,12 @@
       <c r="EX37" s="3">
         <v>127.58084000000001</v>
       </c>
+      <c r="FC37" s="32">
+        <v>105.9058</v>
+      </c>
+      <c r="FD37" s="16"/>
     </row>
-    <row r="38" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="38" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C38" s="7" t="s">
         <v>34</v>
       </c>
@@ -10629,8 +10820,12 @@
       <c r="EY38" s="3">
         <v>155.35636000000002</v>
       </c>
+      <c r="FC38" s="32">
+        <v>96.419066666666666</v>
+      </c>
+      <c r="FD38" s="16"/>
     </row>
-    <row r="39" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="39" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C39" s="7" t="s">
         <v>35</v>
       </c>
@@ -10858,8 +11053,12 @@
       <c r="EZ39" s="3">
         <v>192.77040000000002</v>
       </c>
+      <c r="FC39" s="32">
+        <v>88.801466666666656</v>
+      </c>
+      <c r="FD39" s="16"/>
     </row>
-    <row r="40" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="40" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C40" s="7" t="s">
         <v>36</v>
       </c>
@@ -11090,8 +11289,12 @@
       <c r="FA40" s="3">
         <v>230.90992000000003</v>
       </c>
+      <c r="FC40" s="32">
+        <v>82.488733333333329</v>
+      </c>
+      <c r="FD40" s="16"/>
     </row>
-    <row r="41" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="41" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C41" s="7" t="s">
         <v>37</v>
       </c>
@@ -11340,8 +11543,12 @@
       <c r="FB41" s="3">
         <v>277.13335999999998</v>
       </c>
+      <c r="FC41" s="32">
+        <v>244.76829999999998</v>
+      </c>
+      <c r="FD41" s="16"/>
     </row>
-    <row r="42" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="42" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C42" s="7" t="s">
         <v>38</v>
       </c>
@@ -11590,8 +11797,12 @@
       <c r="FB42" s="3">
         <v>177.22440000000003</v>
       </c>
+      <c r="FC42" s="32">
+        <v>201.17869999999999</v>
+      </c>
+      <c r="FD42" s="16"/>
     </row>
-    <row r="43" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="43" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C43" s="7" t="s">
         <v>39</v>
       </c>
@@ -11855,8 +12066,12 @@
       <c r="FB43" s="3">
         <v>190.69759999999999</v>
       </c>
+      <c r="FC43" s="32">
+        <v>185.15</v>
+      </c>
+      <c r="FD43" s="16"/>
     </row>
-    <row r="44" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="44" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C44" s="7" t="s">
         <v>40</v>
       </c>
@@ -12097,8 +12312,12 @@
       <c r="EW44" s="3">
         <v>81.461040000000011</v>
       </c>
+      <c r="FC44" s="32">
+        <v>174.83449999999999</v>
+      </c>
+      <c r="FD44" s="16"/>
     </row>
-    <row r="45" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="45" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C45" s="7" t="s">
         <v>41</v>
       </c>
@@ -12353,8 +12572,12 @@
       <c r="EY45" s="3">
         <v>125.40440000000001</v>
       </c>
+      <c r="FC45" s="32">
+        <v>167.90459999999999</v>
+      </c>
+      <c r="FD45" s="16"/>
     </row>
-    <row r="46" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="46" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C46" s="7" t="s">
         <v>42</v>
       </c>
@@ -12612,8 +12835,12 @@
       <c r="EZ46" s="3">
         <v>153.38720000000001</v>
       </c>
+      <c r="FC46" s="32">
+        <v>160.18119999999999</v>
+      </c>
+      <c r="FD46" s="16"/>
     </row>
-    <row r="47" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="47" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C47" s="7" t="s">
         <v>43</v>
       </c>
@@ -12853,8 +13080,12 @@
       <c r="EU47" s="3">
         <v>29.537400000000002</v>
       </c>
+      <c r="FC47" s="32">
+        <v>153.67449999999999</v>
+      </c>
+      <c r="FD47" s="16"/>
     </row>
-    <row r="48" spans="3:158" ht="16" x14ac:dyDescent="0.2">
+    <row r="48" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C48" s="7" t="s">
         <v>44</v>
       </c>
@@ -13097,8 +13328,12 @@
       <c r="EU48" s="3">
         <v>28.469908</v>
       </c>
+      <c r="FC48" s="32">
+        <v>152.08750000000001</v>
+      </c>
+      <c r="FD48" s="16"/>
     </row>
-    <row r="49" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="49" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C49" s="7" t="s">
         <v>45</v>
       </c>
@@ -13341,8 +13576,12 @@
       <c r="EU49" s="3">
         <v>31.060908000000001</v>
       </c>
+      <c r="FC49" s="32">
+        <v>149.07220000000001</v>
+      </c>
+      <c r="FD49" s="16"/>
     </row>
-    <row r="50" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="50" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C50" s="7" t="s">
         <v>46</v>
       </c>
@@ -13570,8 +13809,12 @@
       <c r="EU50" s="3">
         <v>32.926428000000001</v>
       </c>
+      <c r="FC50" s="32">
+        <v>58.391020000000005</v>
+      </c>
+      <c r="FD50" s="16"/>
     </row>
-    <row r="51" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="51" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C51" s="7" t="s">
         <v>47</v>
       </c>
@@ -13814,8 +14057,12 @@
       <c r="EU51" s="3">
         <v>34.833404000000002</v>
       </c>
+      <c r="FC51" s="32">
+        <v>144.36410000000001</v>
+      </c>
+      <c r="FD51" s="16"/>
     </row>
-    <row r="52" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="52" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C52" s="7" t="s">
         <v>48</v>
       </c>
@@ -14058,8 +14305,12 @@
       <c r="EU52" s="3">
         <v>37.476224000000002</v>
       </c>
+      <c r="FC52" s="32">
+        <v>130.39849999999998</v>
+      </c>
+      <c r="FD52" s="16"/>
     </row>
-    <row r="53" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="53" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C53" s="7" t="s">
         <v>49</v>
       </c>
@@ -14320,8 +14571,12 @@
       <c r="EV53" s="3">
         <v>53.892800000000008</v>
       </c>
+      <c r="FC53" s="32">
+        <v>152.82809999999998</v>
+      </c>
+      <c r="FD53" s="16"/>
     </row>
-    <row r="54" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="54" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C54" s="7" t="s">
         <v>50</v>
       </c>
@@ -14582,8 +14837,12 @@
       <c r="EW54" s="3">
         <v>72.278536000000003</v>
       </c>
+      <c r="FC54" s="32">
+        <v>137.09916666666666</v>
+      </c>
+      <c r="FD54" s="16"/>
     </row>
-    <row r="55" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="55" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C55" s="7" t="s">
         <v>51</v>
       </c>
@@ -14850,8 +15109,12 @@
       <c r="EX55" s="3">
         <v>107.78560000000002</v>
       </c>
+      <c r="FC55" s="32">
+        <v>124.8969</v>
+      </c>
+      <c r="FD55" s="16"/>
     </row>
-    <row r="56" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="56" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C56" s="7" t="s">
         <v>52</v>
       </c>
@@ -15121,8 +15384,12 @@
       <c r="EY56" s="3">
         <v>136.8048</v>
       </c>
+      <c r="FC56" s="32">
+        <v>115.60413333333332</v>
+      </c>
+      <c r="FD56" s="16"/>
     </row>
-    <row r="57" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="57" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C57" s="7" t="s">
         <v>53</v>
       </c>
@@ -15380,8 +15647,12 @@
       <c r="EU57" s="3">
         <v>33.164800000000007</v>
       </c>
+      <c r="FC57" s="32">
+        <v>107.98653333333333</v>
+      </c>
+      <c r="FD57" s="16"/>
     </row>
-    <row r="58" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="58" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C58" s="7" t="s">
         <v>54</v>
       </c>
@@ -15639,8 +15910,12 @@
       <c r="EV58" s="3">
         <v>32.128400000000006</v>
       </c>
+      <c r="FC58" s="32">
+        <v>101.49746666666668</v>
+      </c>
+      <c r="FD58" s="16"/>
     </row>
-    <row r="59" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="59" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C59" s="7" t="s">
         <v>55</v>
       </c>
@@ -15910,8 +16185,12 @@
       <c r="ET59" s="3">
         <v>23.111720000000002</v>
       </c>
+      <c r="FC59" s="32">
+        <v>271.64150000000001</v>
+      </c>
+      <c r="FD59" s="16"/>
     </row>
-    <row r="60" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="60" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C60" s="7" t="s">
         <v>56</v>
       </c>
@@ -16181,8 +16460,12 @@
       <c r="ET60" s="3">
         <v>10.003954640000002</v>
       </c>
+      <c r="FC60" s="32">
+        <v>227.04679999999999</v>
+      </c>
+      <c r="FD60" s="16"/>
     </row>
-    <row r="61" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="61" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C61" s="7" t="s">
         <v>57</v>
       </c>
@@ -16473,8 +16756,12 @@
       <c r="EW61" s="3">
         <v>49.954480000000004</v>
       </c>
+      <c r="FC61" s="32">
+        <v>210.8065</v>
+      </c>
+      <c r="FD61" s="16"/>
     </row>
-    <row r="62" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="62" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C62" s="7" t="s">
         <v>58</v>
       </c>
@@ -16778,8 +17065,12 @@
       <c r="EW62" s="3">
         <v>36.719652000000004</v>
       </c>
+      <c r="FC62" s="32">
+        <v>207.73830000000001</v>
+      </c>
+      <c r="FD62" s="16"/>
     </row>
-    <row r="63" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="63" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C63" s="7" t="s">
         <v>59</v>
       </c>
@@ -17073,8 +17364,12 @@
       <c r="EX63" s="3">
         <v>57.540928000000001</v>
       </c>
+      <c r="FC63" s="32">
+        <v>214.93269999999998</v>
+      </c>
+      <c r="FD63" s="16"/>
     </row>
-    <row r="64" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="64" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C64" s="7" t="s">
         <v>60</v>
       </c>
@@ -17368,8 +17663,12 @@
       <c r="EX64" s="3">
         <v>60.007560000000005</v>
       </c>
+      <c r="FC64" s="32">
+        <v>211.7587</v>
+      </c>
+      <c r="FD64" s="16"/>
     </row>
-    <row r="65" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="65" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C65" s="7" t="s">
         <v>61</v>
       </c>
@@ -17654,8 +17953,12 @@
       <c r="EX65" s="3">
         <v>61.696892000000005</v>
       </c>
+      <c r="FC65" s="32">
+        <v>208.5318</v>
+      </c>
+      <c r="FD65" s="16"/>
     </row>
-    <row r="66" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="66" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C66" s="7" t="s">
         <v>62</v>
       </c>
@@ -17949,8 +18252,12 @@
       <c r="EX66" s="3">
         <v>62.660744000000008</v>
       </c>
+      <c r="FC66" s="32">
+        <v>205.5694</v>
+      </c>
+      <c r="FD66" s="16"/>
     </row>
-    <row r="67" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="67" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C67" s="7" t="s">
         <v>63</v>
       </c>
@@ -18241,8 +18548,12 @@
       <c r="EX67" s="3">
         <v>63.230764000000008</v>
       </c>
+      <c r="FC67" s="32">
+        <v>202.92439999999999</v>
+      </c>
+      <c r="FD67" s="16"/>
     </row>
-    <row r="68" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="68" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C68" s="7" t="s">
         <v>64</v>
       </c>
@@ -18551,8 +18862,12 @@
       <c r="EX68" s="3">
         <v>64.764635999999996</v>
       </c>
+      <c r="FC68" s="32">
+        <v>190.01679999999999</v>
+      </c>
+      <c r="FD68" s="16"/>
     </row>
-    <row r="69" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="69" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C69" s="7" t="s">
         <v>65</v>
       </c>
@@ -18846,8 +19161,12 @@
       <c r="EX69" s="3">
         <v>66.464332000000013</v>
       </c>
+      <c r="FC69" s="32">
+        <v>197.05250000000001</v>
+      </c>
+      <c r="FD69" s="16"/>
     </row>
-    <row r="70" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="70" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C70" s="7" t="s">
         <v>66</v>
       </c>
@@ -19141,8 +19460,12 @@
       <c r="EX70" s="3">
         <v>62.080360000000006</v>
       </c>
+      <c r="FC70" s="32">
+        <v>194.3546</v>
+      </c>
+      <c r="FD70" s="16"/>
     </row>
-    <row r="71" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="71" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C71" s="7" t="s">
         <v>67</v>
       </c>
@@ -19436,8 +19759,12 @@
       <c r="EX71" s="3">
         <v>63.935516</v>
       </c>
+      <c r="FC71" s="32">
+        <v>191.76249999999999</v>
+      </c>
+      <c r="FD71" s="16"/>
     </row>
-    <row r="72" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="72" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C72" s="7" t="s">
         <v>68</v>
       </c>
@@ -19731,8 +20058,12 @@
       <c r="EX72" s="3">
         <v>65.106648000000007</v>
       </c>
+      <c r="FC72" s="32">
+        <v>189.11750000000001</v>
+      </c>
+      <c r="FD72" s="16"/>
     </row>
-    <row r="73" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="73" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C73" s="7" t="s">
         <v>69</v>
       </c>
@@ -20026,8 +20357,12 @@
       <c r="EX73" s="3">
         <v>65.427931999999998</v>
       </c>
+      <c r="FC73" s="32">
+        <v>186.73699999999999</v>
+      </c>
+      <c r="FD73" s="16"/>
     </row>
-    <row r="74" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="74" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C74" s="7" t="s">
         <v>70</v>
       </c>
@@ -20318,8 +20653,12 @@
       <c r="EX74" s="3">
         <v>65.583392000000003</v>
       </c>
+      <c r="FC74" s="32">
+        <v>184.30359999999999</v>
+      </c>
+      <c r="FD74" s="16"/>
     </row>
-    <row r="75" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="75" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C75" s="7" t="s">
         <v>71</v>
       </c>
@@ -20628,8 +20967,12 @@
       <c r="EX75" s="3">
         <v>66.795980000000014</v>
       </c>
+      <c r="FC75" s="32">
+        <v>170.97280000000001</v>
+      </c>
+      <c r="FD75" s="16"/>
     </row>
-    <row r="76" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="76" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C76" s="7" t="s">
         <v>72</v>
       </c>
@@ -20938,8 +21281,12 @@
       <c r="EX76" s="3">
         <v>68.360944000000003</v>
       </c>
+      <c r="FC76" s="32">
+        <v>162.3501</v>
+      </c>
+      <c r="FD76" s="16"/>
     </row>
-    <row r="77" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="77" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C77" s="7" t="s">
         <v>73</v>
       </c>
@@ -21236,8 +21583,12 @@
       <c r="ES77" s="3">
         <v>7.887004000000001</v>
       </c>
+      <c r="FC77" s="32">
+        <v>155.1028</v>
+      </c>
+      <c r="FD77" s="16"/>
     </row>
-    <row r="78" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="78" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C78" s="7" t="s">
         <v>74</v>
       </c>
@@ -21534,8 +21885,12 @@
       <c r="ES78" s="3">
         <v>7.9802800000000005</v>
       </c>
+      <c r="FC78" s="32">
+        <v>148.86060000000001</v>
+      </c>
+      <c r="FD78" s="16"/>
     </row>
-    <row r="79" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="79" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C79" s="7" t="s">
         <v>75</v>
       </c>
@@ -21832,8 +22187,12 @@
       <c r="ES79" s="3">
         <v>7.876640000000001</v>
       </c>
+      <c r="FC79" s="32">
+        <v>143.41189999999997</v>
+      </c>
+      <c r="FD79" s="16"/>
     </row>
-    <row r="80" spans="3:154" ht="16" x14ac:dyDescent="0.2">
+    <row r="80" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C80" s="7" t="s">
         <v>76</v>
       </c>
@@ -22130,8 +22489,12 @@
       <c r="ES80" s="3">
         <v>8.7057599999999997</v>
       </c>
+      <c r="FC80" s="32">
+        <v>138.06899999999999</v>
+      </c>
+      <c r="FD80" s="16"/>
     </row>
-    <row r="81" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="81" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C81" s="7" t="s">
         <v>77</v>
       </c>
@@ -22428,8 +22791,12 @@
       <c r="ES81" s="3">
         <v>9.1203200000000013</v>
       </c>
+      <c r="FC81" s="32">
+        <v>133.41379999999998</v>
+      </c>
+      <c r="FD81" s="16"/>
     </row>
-    <row r="82" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="82" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C82" s="7" t="s">
         <v>78</v>
       </c>
@@ -22729,8 +23096,12 @@
       <c r="ET82" s="3">
         <v>18.562960400000001</v>
       </c>
+      <c r="FC82" s="32">
+        <v>132.5145</v>
+      </c>
+      <c r="FD82" s="16"/>
     </row>
-    <row r="83" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="83" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C83" s="7" t="s">
         <v>79</v>
       </c>
@@ -23030,8 +23401,12 @@
       <c r="ET83" s="3">
         <v>20.520720000000001</v>
       </c>
+      <c r="FC83" s="32">
+        <v>130.0282</v>
+      </c>
+      <c r="FD83" s="16"/>
     </row>
-    <row r="84" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="84" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C84" s="7" t="s">
         <v>80</v>
       </c>
@@ -23334,8 +23709,12 @@
       <c r="EV84" s="3">
         <v>34.2012</v>
       </c>
+      <c r="FC84" s="32">
+        <v>121.72290000000001</v>
+      </c>
+      <c r="FD84" s="16"/>
     </row>
-    <row r="85" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="85" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C85" s="7" t="s">
         <v>81</v>
       </c>
@@ -23653,8 +24032,12 @@
       <c r="EV85" s="3">
         <v>29.827592000000003</v>
       </c>
+      <c r="FC85" s="32">
+        <v>145.6866</v>
+      </c>
+      <c r="FD85" s="16"/>
     </row>
-    <row r="86" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="86" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C86" s="7" t="s">
         <v>82</v>
       </c>
@@ -23978,8 +24361,12 @@
       <c r="EX86" s="3">
         <v>68.816960000000009</v>
       </c>
+      <c r="FC86" s="32">
+        <v>139.1799</v>
+      </c>
+      <c r="FD86" s="16"/>
     </row>
-    <row r="87" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="87" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C87" s="7" t="s">
         <v>83</v>
       </c>
@@ -24306,8 +24693,12 @@
       <c r="EY87" s="3">
         <v>89.337679999999992</v>
       </c>
+      <c r="FC87" s="32">
+        <v>131.0333</v>
+      </c>
+      <c r="FD87" s="16"/>
     </row>
-    <row r="88" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="88" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C88" s="7" t="s">
         <v>84</v>
       </c>
@@ -24613,8 +25004,12 @@
       <c r="ES88" s="3">
         <v>8.4155680000000004</v>
       </c>
+      <c r="FC88" s="32">
+        <v>122.79853333333334</v>
+      </c>
+      <c r="FD88" s="16"/>
     </row>
-    <row r="89" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="89" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C89" s="7" t="s">
         <v>85</v>
       </c>
@@ -24914,8 +25309,12 @@
         <f t="shared" si="70"/>
         <v>-83.256441680000009</v>
       </c>
+      <c r="FC89" s="32">
+        <v>115.41016666666667</v>
+      </c>
+      <c r="FD89" s="16"/>
     </row>
-    <row r="90" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="90" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C90" s="7" t="s">
         <v>86</v>
       </c>
@@ -25221,8 +25620,12 @@
       <c r="ES90" s="3">
         <v>10.747468</v>
       </c>
+      <c r="FC90" s="32">
+        <v>109.15033333333334</v>
+      </c>
+      <c r="FD90" s="16"/>
     </row>
-    <row r="91" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="91" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C91" s="7" t="s">
         <v>87</v>
       </c>
@@ -25528,8 +25931,12 @@
         <f t="shared" ref="EK91:EK99" si="74">-1*CM91</f>
         <v>-14.277245750000001</v>
       </c>
+      <c r="FC91" s="32">
+        <v>264.07679999999999</v>
+      </c>
+      <c r="FD91" s="16"/>
     </row>
-    <row r="92" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="92" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C92" s="7" t="s">
         <v>88</v>
       </c>
@@ -25850,8 +26257,12 @@
       <c r="ET92" s="3">
         <v>10.146977840000002</v>
       </c>
+      <c r="FC92" s="32">
+        <v>225.2482</v>
+      </c>
+      <c r="FD92" s="16"/>
     </row>
-    <row r="93" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="93" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C93" s="7" t="s">
         <v>89</v>
       </c>
@@ -26190,8 +26601,12 @@
       <c r="ET93" s="3">
         <v>12.12588</v>
       </c>
+      <c r="FC93" s="32">
+        <v>207.42089999999999</v>
+      </c>
+      <c r="FD93" s="16"/>
     </row>
-    <row r="94" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="94" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C94" s="7" t="s">
         <v>90</v>
       </c>
@@ -26539,8 +26954,12 @@
       <c r="EW94" s="3">
         <v>28.811920000000001</v>
       </c>
+      <c r="FC94" s="32">
+        <v>194.8836</v>
+      </c>
+      <c r="FD94" s="16"/>
     </row>
-    <row r="95" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="95" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C95" s="7" t="s">
         <v>91</v>
       </c>
@@ -26891,8 +27310,12 @@
       <c r="ES95" s="3">
         <v>5.9074799999999996</v>
       </c>
+      <c r="FC95" s="32">
+        <v>199.00979999999998</v>
+      </c>
+      <c r="FD95" s="16"/>
     </row>
-    <row r="96" spans="3:155" ht="16" x14ac:dyDescent="0.2">
+    <row r="96" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C96" s="7" t="s">
         <v>92</v>
       </c>
@@ -27246,8 +27669,12 @@
       <c r="ES96" s="3">
         <v>6.1147600000000004</v>
       </c>
+      <c r="FC96" s="32">
+        <v>195.6242</v>
+      </c>
+      <c r="FD96" s="16"/>
     </row>
-    <row r="97" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="97" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C97" s="7" t="s">
         <v>93</v>
       </c>
@@ -27598,8 +28025,12 @@
       <c r="ES97" s="3">
         <v>6.2183999999999999</v>
       </c>
+      <c r="FC97" s="32">
+        <v>192.23859999999999</v>
+      </c>
+      <c r="FD97" s="16"/>
     </row>
-    <row r="98" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="98" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C98" s="7" t="s">
         <v>94</v>
       </c>
@@ -27935,8 +28366,12 @@
       <c r="ES98" s="3">
         <v>6.0629400000000002</v>
       </c>
+      <c r="FC98" s="32">
+        <v>197.74019999999999</v>
+      </c>
+      <c r="FD98" s="16"/>
     </row>
-    <row r="99" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="99" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C99" s="7" t="s">
         <v>95</v>
       </c>
@@ -28272,8 +28707,12 @@
       <c r="ES99" s="3">
         <v>5.9903919999999999</v>
       </c>
+      <c r="FC99" s="32">
+        <v>194.72489999999999</v>
+      </c>
+      <c r="FD99" s="16"/>
     </row>
-    <row r="100" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="100" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C100" s="7" t="s">
         <v>96</v>
       </c>
@@ -28426,8 +28865,12 @@
       <c r="ES100" s="3">
         <v>6.0214840000000001</v>
       </c>
+      <c r="FC100" s="32">
+        <v>182.76949999999999</v>
+      </c>
+      <c r="FD100" s="16"/>
     </row>
-    <row r="101" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="101" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C101" s="7" t="s">
         <v>97</v>
       </c>
@@ -28567,8 +29010,12 @@
       <c r="ES101" s="3">
         <v>6.228764</v>
       </c>
+      <c r="FC101" s="32">
+        <v>188.4298</v>
+      </c>
+      <c r="FD101" s="16"/>
     </row>
-    <row r="102" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="102" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C102" s="7" t="s">
         <v>98</v>
       </c>
@@ -28705,8 +29152,12 @@
       <c r="ES102" s="3">
         <v>6.3013120000000002</v>
       </c>
+      <c r="FC102" s="32">
+        <v>185.57319999999999</v>
+      </c>
+      <c r="FD102" s="16"/>
     </row>
-    <row r="103" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="103" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C103" s="7" t="s">
         <v>99</v>
       </c>
@@ -28843,8 +29294,12 @@
       <c r="ES103" s="3">
         <v>6.4153160000000007</v>
       </c>
+      <c r="FC103" s="32">
+        <v>182.76949999999999</v>
+      </c>
+      <c r="FD103" s="16"/>
     </row>
-    <row r="104" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="104" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C104" s="7" t="s">
         <v>100</v>
       </c>
@@ -28975,8 +29430,12 @@
       <c r="ES104" s="3">
         <v>6.4982280000000001</v>
       </c>
+      <c r="FC104" s="32">
+        <v>179.9658</v>
+      </c>
+      <c r="FD104" s="16"/>
     </row>
-    <row r="105" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="105" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C105" s="7" t="s">
         <v>101</v>
       </c>
@@ -29107,8 +29566,12 @@
       <c r="ES105" s="3">
         <v>6.5811400000000004</v>
       </c>
+      <c r="FC105" s="32">
+        <v>177.37370000000001</v>
+      </c>
+      <c r="FD105" s="16"/>
     </row>
-    <row r="106" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="106" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C106" s="7" t="s">
         <v>102</v>
       </c>
@@ -29239,8 +29702,12 @@
       <c r="ES106" s="3">
         <v>6.6536880000000007</v>
       </c>
+      <c r="FC106" s="32">
+        <v>174.83449999999999</v>
+      </c>
+      <c r="FD106" s="16"/>
     </row>
-    <row r="107" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="107" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C107" s="7" t="s">
         <v>103</v>
       </c>
@@ -29372,8 +29839,12 @@
       <c r="BH107" s="24">
         <v>201.70770000000002</v>
       </c>
+      <c r="FC107" s="32">
+        <v>201.70770000000002</v>
+      </c>
+      <c r="FD107" s="16"/>
     </row>
-    <row r="108" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="108" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C108" s="7" t="s">
         <v>104</v>
       </c>
@@ -29499,8 +29970,12 @@
         <v>153.30420000000001</v>
       </c>
       <c r="BH108" s="24"/>
+      <c r="FC108" s="32">
+        <v>153.30420000000001</v>
+      </c>
+      <c r="FD108" s="16"/>
     </row>
-    <row r="109" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="109" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C109" s="7" t="s">
         <v>105</v>
       </c>
@@ -29626,8 +30101,12 @@
         <v>145.9511</v>
       </c>
       <c r="BH109" s="24"/>
+      <c r="FC109" s="32">
+        <v>145.9511</v>
+      </c>
+      <c r="FD109" s="16"/>
     </row>
-    <row r="110" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="110" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C110" s="7" t="s">
         <v>106</v>
       </c>
@@ -29753,8 +30232,12 @@
         <v>139.86760000000001</v>
       </c>
       <c r="BH110" s="24"/>
+      <c r="FC110" s="32">
+        <v>139.86760000000001</v>
+      </c>
+      <c r="FD110" s="16"/>
     </row>
-    <row r="111" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="111" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C111" s="7" t="s">
         <v>107</v>
       </c>
@@ -29880,8 +30363,12 @@
         <v>133.14929999999998</v>
       </c>
       <c r="BH111" s="24"/>
+      <c r="FC111" s="32">
+        <v>133.14929999999998</v>
+      </c>
+      <c r="FD111" s="16"/>
     </row>
-    <row r="112" spans="3:149" ht="16" x14ac:dyDescent="0.2">
+    <row r="112" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C112" s="7" t="s">
         <v>108</v>
       </c>
@@ -30007,8 +30494,12 @@
         <v>128.12380000000002</v>
       </c>
       <c r="BH112" s="24"/>
+      <c r="FC112" s="32">
+        <v>128.12380000000002</v>
+      </c>
+      <c r="FD112" s="16"/>
     </row>
-    <row r="113" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="113" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C113" s="7" t="s">
         <v>109</v>
       </c>
@@ -30134,8 +30625,12 @@
         <v>123.15119999999999</v>
       </c>
       <c r="BH113" s="24"/>
+      <c r="FC113" s="32">
+        <v>123.15119999999999</v>
+      </c>
+      <c r="FD113" s="16"/>
     </row>
-    <row r="114" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="114" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C114" s="7" t="s">
         <v>110</v>
       </c>
@@ -30261,8 +30756,12 @@
         <v>119.4482</v>
       </c>
       <c r="BH114" s="24"/>
+      <c r="FC114" s="32">
+        <v>119.4482</v>
+      </c>
+      <c r="FD114" s="16"/>
     </row>
-    <row r="115" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="115" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C115" s="7" t="s">
         <v>111</v>
       </c>
@@ -30388,8 +30887,12 @@
         <v>116.38000000000001</v>
       </c>
       <c r="BH115" s="24"/>
+      <c r="FC115" s="32">
+        <v>116.38000000000001</v>
+      </c>
+      <c r="FD115" s="16"/>
     </row>
-    <row r="116" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="116" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C116" s="7" t="s">
         <v>112</v>
       </c>
@@ -30515,8 +31018,12 @@
         <v>111.30160000000001</v>
       </c>
       <c r="BH116" s="24"/>
+      <c r="FC116" s="32">
+        <v>111.30160000000001</v>
+      </c>
+      <c r="FD116" s="16"/>
     </row>
-    <row r="117" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="117" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C117" s="7" t="s">
         <v>113</v>
       </c>
@@ -30646,8 +31153,12 @@
       <c r="BH117" s="24">
         <v>128.2825</v>
       </c>
+      <c r="FC117" s="32">
+        <v>128.2825</v>
+      </c>
+      <c r="FD117" s="16"/>
     </row>
-    <row r="118" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="118" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C118" s="7" t="s">
         <v>114</v>
       </c>
@@ -30777,8 +31288,12 @@
       <c r="BH118" s="24">
         <v>135.19476666666665</v>
       </c>
+      <c r="FC118" s="32">
+        <v>135.19476666666665</v>
+      </c>
+      <c r="FD118" s="16"/>
     </row>
-    <row r="119" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="119" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C119" s="7" t="s">
         <v>115</v>
       </c>
@@ -30908,8 +31423,12 @@
       <c r="BH119" s="24">
         <v>140.97849999999997</v>
       </c>
+      <c r="FC119" s="32">
+        <v>140.97849999999997</v>
+      </c>
+      <c r="FD119" s="16"/>
     </row>
-    <row r="120" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="120" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C120" s="7" t="s">
         <v>116</v>
       </c>
@@ -31039,8 +31558,12 @@
       <c r="BH120" s="24">
         <v>133.69593333333333</v>
       </c>
+      <c r="FC120" s="32">
+        <v>133.69593333333333</v>
+      </c>
+      <c r="FD120" s="16"/>
     </row>
-    <row r="121" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="121" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C121" s="7" t="s">
         <v>117</v>
       </c>
@@ -31170,8 +31693,12 @@
       <c r="BH121" s="24">
         <v>123.36280000000001</v>
       </c>
+      <c r="FC121" s="32">
+        <v>123.36280000000001</v>
+      </c>
+      <c r="FD121" s="16"/>
     </row>
-    <row r="122" spans="3:142" ht="16" x14ac:dyDescent="0.2">
+    <row r="122" spans="3:160" ht="16" x14ac:dyDescent="0.2">
       <c r="C122" s="7" t="s">
         <v>118</v>
       </c>
@@ -31510,8 +32037,12 @@
         <f t="shared" si="79"/>
         <v>-125.271584</v>
       </c>
+      <c r="FC122" s="32">
+        <v>118.7076</v>
+      </c>
+      <c r="FD122" s="16"/>
     </row>
-    <row r="123" spans="3:142" x14ac:dyDescent="0.2">
+    <row r="123" spans="3:160" x14ac:dyDescent="0.2">
       <c r="K123" s="28"/>
       <c r="L123" s="28"/>
       <c r="M123" s="28"/>
@@ -31534,6 +32065,8 @@
     </row>
   </sheetData>
   <mergeCells count="33">
+    <mergeCell ref="DN2:DS2"/>
+    <mergeCell ref="EM1:ER1"/>
     <mergeCell ref="ES2:FB2"/>
     <mergeCell ref="ES4:FB4"/>
     <mergeCell ref="AP4:BH4"/>
@@ -31549,7 +32082,7 @@
     <mergeCell ref="CO4:CT4"/>
     <mergeCell ref="BI4:BN4"/>
     <mergeCell ref="BI2:BN2"/>
-    <mergeCell ref="DN2:DS2"/>
+    <mergeCell ref="ES1:FB1"/>
     <mergeCell ref="EM2:ER2"/>
     <mergeCell ref="EM4:ER4"/>
     <mergeCell ref="K1:AC1"/>
@@ -31565,8 +32098,6 @@
     <mergeCell ref="CU1:DM1"/>
     <mergeCell ref="DN1:DS1"/>
     <mergeCell ref="DT1:EL1"/>
-    <mergeCell ref="EM1:ER1"/>
-    <mergeCell ref="ES1:FB1"/>
   </mergeCells>
   <phoneticPr fontId="7" type="noConversion"/>
   <hyperlinks>
@@ -31580,6 +32111,7 @@
     <hyperlink ref="BR1" r:id="rId8" xr:uid="{41EBA78A-472B-4079-A7E6-B09F91178D2A}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <legacyDrawing r:id="rId9"/>
 </worksheet>
 </file>
</xml_diff>